<commit_message>
Updates data files with latest information
Updates several data files to reflect the latest changes and corrections.

These files contain important information related to products and offers,
and keeping them up-to-date ensures data accuracy and consistency.
</commit_message>
<xml_diff>
--- a/dados_produtos_corrigidos.xlsx
+++ b/dados_produtos_corrigidos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E530"/>
+  <dimension ref="A1:E532"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11756,6 +11756,52 @@
         <v>55.99</v>
       </c>
     </row>
+    <row r="531">
+      <c r="A531" t="n">
+        <v>105450</v>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>#06 AÇOUGUE - BOVINO</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>BOVINO - ALCATRA KG</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>ALCATRA BOVINA KG</t>
+        </is>
+      </c>
+      <c r="E531" t="n">
+        <v>37.99</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="n">
+        <v>105456</v>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>#06 AÇOUGUE - BOVINO</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>BOVINO - CARNE DE SOL KG SEGUNDA</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>CARNE DE SOL KG SEGUNDA</t>
+        </is>
+      </c>
+      <c r="E532" t="n">
+        <v>26.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updates data files with corrected information
Updates the data files to reflect corrected and consolidated information related to products and offers.
</commit_message>
<xml_diff>
--- a/dados_produtos_corrigidos.xlsx
+++ b/dados_produtos_corrigidos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E593"/>
+  <dimension ref="A1:E595"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13205,6 +13205,52 @@
         <v>9.49</v>
       </c>
     </row>
+    <row r="594">
+      <c r="A594" t="n">
+        <v>104855</v>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>#09 HORTIFRUTI</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>LIMAO TAITI KG</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>LIMAO TAITI KG</t>
+        </is>
+      </c>
+      <c r="E594" t="n">
+        <v>4.69</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="n">
+        <v>104962</v>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>#09 HORTIFRUTI</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>MARACUJA AZEDO</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>MARACUJA AZEDO KG</t>
+        </is>
+      </c>
+      <c r="E595" t="n">
+        <v>4.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>